<commit_message>
actualizacion formatos y rutas en main
</commit_message>
<xml_diff>
--- a/BD_airtable.xlsx
+++ b/BD_airtable.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/078e1a455e5c02ce/Documentos/GitHub/Proyecto_PIPC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="80" documentId="8_{B145F242-E461-4697-BC30-B63A2CA7B06A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7E1C40B7-260D-497A-9E62-2DF9795E8349}"/>
+  <xr:revisionPtr revIDLastSave="82" documentId="8_{B145F242-E461-4697-BC30-B63A2CA7B06A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6014B0AB-7D94-47D0-9778-E21CAD0DC9D3}"/>
   <bookViews>
-    <workbookView xWindow="13728" yWindow="0" windowWidth="9408" windowHeight="12336" activeTab="2" xr2:uid="{3F095A75-F066-4695-8672-8D4315F1EF23}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{3F095A75-F066-4695-8672-8D4315F1EF23}"/>
   </bookViews>
   <sheets>
     <sheet name="BD" sheetId="1" r:id="rId1"/>
@@ -8848,7 +8848,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
@@ -8870,7 +8870,6 @@
     <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -52453,7 +52452,7 @@
       <c r="J50" s="16" t="s">
         <v>179</v>
       </c>
-      <c r="K50" s="1" t="s">
+      <c r="K50" s="6" t="s">
         <v>268</v>
       </c>
       <c r="L50" t="str">
@@ -52497,7 +52496,7 @@
       <c r="J51" s="16" t="s">
         <v>396</v>
       </c>
-      <c r="K51" s="1" t="s">
+      <c r="K51" s="6" t="s">
         <v>397</v>
       </c>
       <c r="L51" t="str">
@@ -52541,7 +52540,7 @@
       <c r="J52" s="16" t="s">
         <v>181</v>
       </c>
-      <c r="K52" s="1" t="s">
+      <c r="K52" s="6" t="s">
         <v>270</v>
       </c>
       <c r="L52" t="str">
@@ -54346,7 +54345,7 @@
       <c r="J95" s="16" t="s">
         <v>190</v>
       </c>
-      <c r="K95" s="1" t="s">
+      <c r="K95" s="6" t="s">
         <v>300</v>
       </c>
       <c r="L95" t="str">
@@ -54386,7 +54385,7 @@
       <c r="J96" s="16" t="s">
         <v>191</v>
       </c>
-      <c r="K96" s="1" t="s">
+      <c r="K96" s="6" t="s">
         <v>301</v>
       </c>
       <c r="L96" t="str">
@@ -54426,7 +54425,7 @@
       <c r="J97" s="16" t="s">
         <v>192</v>
       </c>
-      <c r="K97" s="1" t="s">
+      <c r="K97" s="6" t="s">
         <v>302</v>
       </c>
       <c r="L97" t="str">
@@ -54466,7 +54465,7 @@
       <c r="J98" s="16" t="s">
         <v>193</v>
       </c>
-      <c r="K98" s="1" t="s">
+      <c r="K98" s="6" t="s">
         <v>303</v>
       </c>
       <c r="L98" t="str">
@@ -55695,7 +55694,7 @@
       <c r="J138" s="18" t="s">
         <v>211</v>
       </c>
-      <c r="K138" s="21" t="s">
+      <c r="K138" t="s">
         <v>324</v>
       </c>
       <c r="L138" t="str">
@@ -55731,7 +55730,7 @@
       <c r="J141" s="18" t="s">
         <v>214</v>
       </c>
-      <c r="K141" s="21" t="s">
+      <c r="K141" t="s">
         <v>327</v>
       </c>
       <c r="L141" t="str">
@@ -55767,7 +55766,7 @@
       <c r="J144" s="18" t="s">
         <v>217</v>
       </c>
-      <c r="K144" s="21" t="s">
+      <c r="K144" t="s">
         <v>330</v>
       </c>
       <c r="L144" t="str">
@@ -55803,7 +55802,7 @@
       <c r="J147" s="18" t="s">
         <v>220</v>
       </c>
-      <c r="K147" s="21" t="s">
+      <c r="K147" t="s">
         <v>333</v>
       </c>
       <c r="L147" t="str">

</xml_diff>